<commit_message>
fixed bug: warning message not printing with messy source data
</commit_message>
<xml_diff>
--- a/inst/extdata/a3_2025_modified.xlsx
+++ b/inst/extdata/a3_2025_modified.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ernestcaballero/Developer/data501/peridial/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E58DB4D-1D35-074F-A215-E2F13F36BAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2634D6AF-CFAD-264F-AD25-6588186DB30C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2984,18 +2984,14 @@
       <c r="L54" s="2">
         <v>44430</v>
       </c>
-      <c r="M54" s="2">
-        <v>45950</v>
-      </c>
+      <c r="M54" s="2"/>
       <c r="N54" t="s">
         <v>88</v>
       </c>
       <c r="O54" t="s">
         <v>28</v>
       </c>
-      <c r="S54" s="2">
-        <v>45950</v>
-      </c>
+      <c r="S54" s="2"/>
       <c r="T54" t="s">
         <v>89</v>
       </c>
@@ -3299,9 +3295,7 @@
       <c r="L60" s="2">
         <v>45330</v>
       </c>
-      <c r="M60" s="2">
-        <v>45807</v>
-      </c>
+      <c r="M60" s="2"/>
       <c r="N60" t="s">
         <v>105</v>
       </c>

</xml_diff>